<commit_message>
04.1: remove duplicate T076 trace; 04.2 codebook revision 1.2; 04.3: rebuild convergent-set flags from 03.2
</commit_message>
<xml_diff>
--- a/materials/04_rg_intervention_framework/asb_framework_04_1_rg_intervention_framework.xlsx
+++ b/materials/04_rg_intervention_framework/asb_framework_04_1_rg_intervention_framework.xlsx
@@ -6492,7 +6492,7 @@
       </c>
       <c r="L83" s="80" t="inlineStr">
         <is>
-          <t>EXP_2016_Auer_FEED-PERSONAL, OBS_2023_Auer_CONTACT-WRITTEN, OBS_2023_Auer_CONTACT-WRITTEN</t>
+          <t>EXP_2016_Auer_FEED-PERSONAL, OBS_2023_Auer_CONTACT-WRITTEN</t>
         </is>
       </c>
       <c r="M83" s="80" t="inlineStr">
@@ -6772,7 +6772,7 @@
     <row r="88" ht="26" customHeight="1">
       <c r="A88" s="61" t="inlineStr">
         <is>
-          <t>▶  PERSONALIZED FEEDBACK</t>
+          <t>▶  PERSONALISED FEEDBACK</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6784,7 @@
       </c>
       <c r="B89" s="82" t="inlineStr">
         <is>
-          <t>Personalized Feedback</t>
+          <t>Personalised Feedback</t>
         </is>
       </c>
       <c r="C89" s="82" t="inlineStr">
@@ -6851,7 +6851,7 @@
       </c>
       <c r="B90" s="83" t="inlineStr">
         <is>
-          <t>Personalized Feedback</t>
+          <t>Personalised Feedback</t>
         </is>
       </c>
       <c r="C90" s="83" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="B91" s="82" t="inlineStr">
         <is>
-          <t>Personalized Feedback</t>
+          <t>Personalised Feedback</t>
         </is>
       </c>
       <c r="C91" s="82" t="inlineStr">
@@ -6985,7 +6985,7 @@
       </c>
       <c r="B92" s="83" t="inlineStr">
         <is>
-          <t>Personalized Feedback</t>
+          <t>Personalised Feedback</t>
         </is>
       </c>
       <c r="C92" s="83" t="inlineStr">
@@ -7052,7 +7052,7 @@
       </c>
       <c r="B93" s="82" t="inlineStr">
         <is>
-          <t>Personalized Feedback</t>
+          <t>Personalised Feedback</t>
         </is>
       </c>
       <c r="C93" s="82" t="inlineStr">
@@ -7119,7 +7119,7 @@
       </c>
       <c r="B94" s="83" t="inlineStr">
         <is>
-          <t>Personalized Feedback</t>
+          <t>Personalised Feedback</t>
         </is>
       </c>
       <c r="C94" s="83" t="inlineStr">
@@ -7186,7 +7186,7 @@
       </c>
       <c r="B95" s="82" t="inlineStr">
         <is>
-          <t>Personalized Feedback</t>
+          <t>Personalised Feedback</t>
         </is>
       </c>
       <c r="C95" s="82" t="inlineStr">
@@ -7253,7 +7253,7 @@
       </c>
       <c r="B96" s="83" t="inlineStr">
         <is>
-          <t>Personalized Feedback</t>
+          <t>Personalised Feedback</t>
         </is>
       </c>
       <c r="C96" s="83" t="inlineStr">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="B97" s="82" t="inlineStr">
         <is>
-          <t>Personalized Feedback</t>
+          <t>Personalised Feedback</t>
         </is>
       </c>
       <c r="C97" s="82" t="inlineStr">
@@ -15365,8 +15365,8 @@
     <mergeCell ref="A98:M98"/>
     <mergeCell ref="A177:M177"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A150:M150"/>
     <mergeCell ref="A133:M133"/>
-    <mergeCell ref="A150:M150"/>
     <mergeCell ref="A106:M106"/>
     <mergeCell ref="A161:M161"/>
     <mergeCell ref="A88:M88"/>

</xml_diff>